<commit_message>
Remove contribution split section (incomes close enough)
</commit_message>
<xml_diff>
--- a/01-current-budget/current-budget.xlsx
+++ b/01-current-budget/current-budget.xlsx
@@ -128,9 +128,9 @@
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E74"/>
+  <dimension ref="A1:E69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -597,388 +597,382 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>2. Contribution Split (optional — for shared costs)</t>
+          <t>2. Fixed Needs — target ~50% of income</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr"/>
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Kate</t>
+          <t>Monthly Amount</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Lucas</t>
+          <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>% of combined income</t>
-        </is>
-      </c>
-      <c r="B12" s="11">
-        <f>IFERROR(B8/$D$8,0)</f>
-        <v/>
-      </c>
-      <c r="C12" s="11">
-        <f>IFERROR(C8/$D$8,0)</f>
-        <v/>
-      </c>
+          <t>Rent / mortgage</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="n"/>
+      <c r="C12" s="11" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="inlineStr">
-        <is>
-          <t>Use this to split shared bills proportionally instead of 50/50, if incomes differ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>3. Fixed Needs — target ~50% of income</t>
-        </is>
-      </c>
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Renters or homeowners insurance</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="n"/>
+      <c r="C13" s="11" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Electricity / gas / water</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="n"/>
+      <c r="C14" s="11" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Internet</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="n"/>
+      <c r="C15" s="11" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>Monthly Amount</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Phone (both lines)</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="n"/>
+      <c r="C16" s="11" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Rent / mortgage</t>
+          <t>Health insurance (if not payroll-deducted)</t>
         </is>
       </c>
       <c r="B17" s="7" t="n"/>
-      <c r="C17" s="13" t="n"/>
+      <c r="C17" s="11" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Renters or homeowners insurance</t>
+          <t>Auto insurance</t>
         </is>
       </c>
       <c r="B18" s="7" t="n"/>
-      <c r="C18" s="13" t="n"/>
+      <c r="C18" s="11" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Electricity / gas / water</t>
+          <t>Car payment(s)</t>
         </is>
       </c>
       <c r="B19" s="7" t="n"/>
-      <c r="C19" s="13" t="n"/>
+      <c r="C19" s="11" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Internet</t>
+          <t>Gas / transit / rideshare (commuting)</t>
         </is>
       </c>
       <c r="B20" s="7" t="n"/>
-      <c r="C20" s="13" t="n"/>
+      <c r="C20" s="11" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>Phone (both lines)</t>
+          <t>Groceries</t>
         </is>
       </c>
       <c r="B21" s="7" t="n"/>
-      <c r="C21" s="13" t="n"/>
+      <c r="C21" s="11" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>Health insurance (if not payroll-deducted)</t>
+          <t>Minimum debt payments (student loans, credit cards, etc.)</t>
         </is>
       </c>
       <c r="B22" s="7" t="n"/>
-      <c r="C22" s="13" t="n"/>
+      <c r="C22" s="11" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Auto insurance</t>
+          <t>Childcare / pet care (if applicable)</t>
         </is>
       </c>
       <c r="B23" s="7" t="n"/>
-      <c r="C23" s="13" t="n"/>
+      <c r="C23" s="11" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t>Car payment(s)</t>
-        </is>
-      </c>
-      <c r="B24" s="7" t="n"/>
-      <c r="C24" s="13" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>Gas / transit / rideshare (commuting)</t>
-        </is>
-      </c>
-      <c r="B25" s="7" t="n"/>
-      <c r="C25" s="13" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="6" t="inlineStr">
-        <is>
-          <t>Groceries</t>
-        </is>
-      </c>
-      <c r="B26" s="7" t="n"/>
-      <c r="C26" s="13" t="n"/>
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>Subtotal — Needs</t>
+        </is>
+      </c>
+      <c r="B24" s="10">
+        <f>SUM(B12:B23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>3. Savings &amp; Goals — zero-based, prioritize explicitly</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="inlineStr">
-        <is>
-          <t>Minimum debt payments (student loans, credit cards, etc.)</t>
-        </is>
-      </c>
-      <c r="B27" s="7" t="n"/>
-      <c r="C27" s="13" t="n"/>
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Monthly Amount</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>Childcare / pet care (if applicable)</t>
+          <t>401(k) / retirement contributions (Kate)</t>
         </is>
       </c>
       <c r="B28" s="7" t="n"/>
-      <c r="C28" s="13" t="n"/>
+      <c r="C28" s="11" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="9" t="inlineStr">
-        <is>
-          <t>Subtotal — Needs</t>
-        </is>
-      </c>
-      <c r="B29" s="10">
-        <f>SUM(B17:B28)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="3" t="inlineStr">
-        <is>
-          <t>4. Savings &amp; Goals — zero-based, prioritize explicitly</t>
-        </is>
-      </c>
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>401(k) / retirement contributions (Lucas)</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="n"/>
+      <c r="C29" s="11" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>Emergency fund</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="n"/>
+      <c r="C30" s="11" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>House down payment fund (Portland)</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="n"/>
+      <c r="C31" s="11" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="B32" s="5" t="inlineStr">
-        <is>
-          <t>Monthly Amount</t>
-        </is>
-      </c>
-      <c r="C32" s="5" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>Wedding fund</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="n"/>
+      <c r="C32" s="11" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>401(k) / retirement contributions (Kate)</t>
+          <t>Other investments</t>
         </is>
       </c>
       <c r="B33" s="7" t="n"/>
-      <c r="C33" s="13" t="n"/>
+      <c r="C33" s="11" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>401(k) / retirement contributions (Lucas)</t>
+          <t>Extra debt paydown (beyond minimums)</t>
         </is>
       </c>
       <c r="B34" s="7" t="n"/>
-      <c r="C34" s="13" t="n"/>
+      <c r="C34" s="11" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="6" t="inlineStr">
-        <is>
-          <t>Emergency fund</t>
-        </is>
-      </c>
-      <c r="B35" s="7" t="n"/>
-      <c r="C35" s="13" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="6" t="inlineStr">
-        <is>
-          <t>House down payment fund (Portland)</t>
-        </is>
-      </c>
-      <c r="B36" s="7" t="n"/>
-      <c r="C36" s="13" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="6" t="inlineStr">
-        <is>
-          <t>Wedding fund</t>
-        </is>
-      </c>
-      <c r="B37" s="7" t="n"/>
-      <c r="C37" s="13" t="n"/>
+      <c r="A35" s="9" t="inlineStr">
+        <is>
+          <t>Subtotal — Savings &amp; Goals</t>
+        </is>
+      </c>
+      <c r="B35" s="10">
+        <f>SUM(B28:B34)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>4. Wants / Discretionary (shared) — target ~30% of income</t>
+        </is>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" s="6" t="inlineStr">
-        <is>
-          <t>Other investments</t>
-        </is>
-      </c>
-      <c r="B38" s="7" t="n"/>
-      <c r="C38" s="13" t="n"/>
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>Monthly Amount</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>Extra debt paydown (beyond minimums)</t>
+          <t>Dining out / takeout</t>
         </is>
       </c>
       <c r="B39" s="7" t="n"/>
-      <c r="C39" s="13" t="n"/>
+      <c r="C39" s="11" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="9" t="inlineStr">
-        <is>
-          <t>Subtotal — Savings &amp; Goals</t>
-        </is>
-      </c>
-      <c r="B40" s="10">
-        <f>SUM(B33:B39)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42" ht="20" customHeight="1">
-      <c r="A42" s="3" t="inlineStr">
-        <is>
-          <t>5. Wants / Discretionary (shared) — target ~30% of income</t>
-        </is>
-      </c>
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>Entertainment &amp; experiences (movies, concerts, hobbies, outings)</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="n"/>
+      <c r="C40" s="11" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>Subscriptions (streaming, apps, memberships)</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="n"/>
+      <c r="C41" s="11" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>Travel / vacation (monthly average)</t>
+        </is>
+      </c>
+      <c r="B42" s="7" t="n"/>
+      <c r="C42" s="11" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="4" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="B43" s="5" t="inlineStr">
-        <is>
-          <t>Monthly Amount</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>Gifts (holidays, birthdays, etc.)</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="n"/>
+      <c r="C43" s="11" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>Dining out / takeout</t>
+          <t>Shopping (clothes, household goods)</t>
         </is>
       </c>
       <c r="B44" s="7" t="n"/>
-      <c r="C44" s="13" t="n"/>
+      <c r="C44" s="11" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>Entertainment &amp; experiences (movies, concerts, hobbies, outings)</t>
+          <t>Personal care (haircuts, gym, etc. — shared/household level)</t>
         </is>
       </c>
       <c r="B45" s="7" t="n"/>
-      <c r="C45" s="13" t="n"/>
+      <c r="C45" s="11" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="6" t="inlineStr">
-        <is>
-          <t>Subscriptions (streaming, apps, memberships)</t>
-        </is>
-      </c>
-      <c r="B46" s="7" t="n"/>
-      <c r="C46" s="13" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="6" t="inlineStr">
-        <is>
-          <t>Travel / vacation (monthly average)</t>
-        </is>
-      </c>
-      <c r="B47" s="7" t="n"/>
-      <c r="C47" s="13" t="n"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="6" t="inlineStr">
-        <is>
-          <t>Gifts (holidays, birthdays, etc.)</t>
-        </is>
-      </c>
-      <c r="B48" s="7" t="n"/>
-      <c r="C48" s="13" t="n"/>
+      <c r="A46" s="9" t="inlineStr">
+        <is>
+          <t>Subtotal — Shared Wants</t>
+        </is>
+      </c>
+      <c r="B46" s="10">
+        <f>SUM(B39:B45)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48" ht="20" customHeight="1">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>5. Individual "Fun Money" — no itemizing, no questions asked</t>
+        </is>
+      </c>
     </row>
     <row r="49">
-      <c r="A49" s="6" t="inlineStr">
-        <is>
-          <t>Shopping (clothes, household goods)</t>
-        </is>
-      </c>
-      <c r="B49" s="7" t="n"/>
-      <c r="C49" s="13" t="n"/>
+      <c r="A49" s="4" t="inlineStr"/>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>Kate</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>Lucas</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>Personal care (haircuts, gym, etc. — shared/household level)</t>
+          <t>Monthly personal allowance</t>
         </is>
       </c>
       <c r="B50" s="7" t="n"/>
-      <c r="C50" s="13" t="n"/>
+      <c r="C50" s="7" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="9" t="inlineStr">
-        <is>
-          <t>Subtotal — Shared Wants</t>
-        </is>
-      </c>
-      <c r="B51" s="10">
-        <f>SUM(B44:B50)</f>
-        <v/>
+      <c r="A51" s="12" t="inlineStr">
+        <is>
+          <t>This is the one category each of you spends freely without justifying to the other.</t>
+        </is>
       </c>
     </row>
     <row r="53" ht="20" customHeight="1">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>6. Individual "Fun Money" — no itemizing, no questions asked</t>
+          <t>6. Zero-Based Check</t>
         </is>
       </c>
     </row>
@@ -986,225 +980,187 @@
       <c r="A54" s="4" t="inlineStr"/>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>Kate</t>
-        </is>
-      </c>
-      <c r="C54" s="5" t="inlineStr">
-        <is>
-          <t>Lucas</t>
+          <t>Amount</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>Monthly personal allowance</t>
-        </is>
-      </c>
-      <c r="B55" s="7" t="n"/>
-      <c r="C55" s="7" t="n"/>
+          <t>Total combined income (Section 1)</t>
+        </is>
+      </c>
+      <c r="B55" s="8">
+        <f>D8</f>
+        <v/>
+      </c>
     </row>
     <row r="56">
-      <c r="A56" s="12" t="inlineStr">
-        <is>
-          <t>This is the one category each of you spends freely without justifying to the other.</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="20" customHeight="1">
-      <c r="A58" s="3" t="inlineStr">
-        <is>
-          <t>7. Zero-Based Check</t>
-        </is>
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t>minus Needs (Section 2 subtotal)</t>
+        </is>
+      </c>
+      <c r="B56" s="8">
+        <f>-B24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="inlineStr">
+        <is>
+          <t>minus Savings &amp; Goals (Section 3 subtotal)</t>
+        </is>
+      </c>
+      <c r="B57" s="8">
+        <f>-B35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>minus Shared Wants (Section 4 subtotal)</t>
+        </is>
+      </c>
+      <c r="B58" s="8">
+        <f>-B46</f>
+        <v/>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="4" t="inlineStr"/>
-      <c r="B59" s="5" t="inlineStr">
-        <is>
-          <t>Amount</t>
-        </is>
+      <c r="A59" s="6" t="inlineStr">
+        <is>
+          <t>minus Fun Money (Section 5, both people)</t>
+        </is>
+      </c>
+      <c r="B59" s="8">
+        <f>-(B50+C50)</f>
+        <v/>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="6" t="inlineStr">
-        <is>
-          <t>Total combined income (Section 1)</t>
-        </is>
-      </c>
-      <c r="B60" s="8">
-        <f>D8</f>
+      <c r="A60" s="9" t="inlineStr">
+        <is>
+          <t>Unassigned (should be $0)</t>
+        </is>
+      </c>
+      <c r="B60" s="10">
+        <f>SUM(B55:B59)</f>
         <v/>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="6" t="inlineStr">
-        <is>
-          <t>minus Needs (Section 3 subtotal)</t>
-        </is>
-      </c>
-      <c r="B61" s="8">
-        <f>-B29</f>
-        <v/>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="6" t="inlineStr">
-        <is>
-          <t>minus Savings &amp; Goals (Section 4 subtotal)</t>
-        </is>
-      </c>
-      <c r="B62" s="8">
-        <f>-B40</f>
-        <v/>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="6" t="inlineStr">
-        <is>
-          <t>minus Shared Wants (Section 5 subtotal)</t>
-        </is>
-      </c>
-      <c r="B63" s="8">
-        <f>-B51</f>
-        <v/>
+      <c r="A61" s="12" t="inlineStr">
+        <is>
+          <t>Negative = cut something (usually Section 4). Positive = assign the leftover, most likely to Section 3 (house/wedding funds).</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="20" customHeight="1">
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t>7. Quick 50/30/20 Sanity Check (optional)</t>
+        </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="6" t="inlineStr">
-        <is>
-          <t>minus Fun Money (Section 6, both people)</t>
-        </is>
-      </c>
-      <c r="B64" s="8">
-        <f>-(B55+C55)</f>
-        <v/>
+      <c r="A64" s="4" t="inlineStr">
+        <is>
+          <t>Bucket</t>
+        </is>
+      </c>
+      <c r="B64" s="5" t="inlineStr">
+        <is>
+          <t>Target %</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="inlineStr">
+        <is>
+          <t>Your %</t>
+        </is>
+      </c>
+      <c r="D64" s="5" t="inlineStr">
+        <is>
+          <t>Your $</t>
+        </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="9" t="inlineStr">
-        <is>
-          <t>Unassigned (should be $0)</t>
-        </is>
-      </c>
-      <c r="B65" s="10">
-        <f>SUM(B60:B64)</f>
+      <c r="A65" s="6" t="inlineStr">
+        <is>
+          <t>Needs (Section 2)</t>
+        </is>
+      </c>
+      <c r="B65" s="13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C65" s="13">
+        <f>IFERROR(D65/D8,0)</f>
+        <v/>
+      </c>
+      <c r="D65" s="8">
+        <f>B24</f>
         <v/>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="12" t="inlineStr">
-        <is>
-          <t>Negative = cut something (usually Section 5). Positive = assign the leftover, most likely to Section 4 (house/wedding funds).</t>
-        </is>
-      </c>
-    </row>
-    <row r="68" ht="20" customHeight="1">
-      <c r="A68" s="3" t="inlineStr">
-        <is>
-          <t>8. Quick 50/30/20 Sanity Check (optional)</t>
-        </is>
+      <c r="A66" s="6" t="inlineStr">
+        <is>
+          <t>Wants (Sections 4 + 5)</t>
+        </is>
+      </c>
+      <c r="B66" s="13" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C66" s="13">
+        <f>IFERROR(D66/D8,0)</f>
+        <v/>
+      </c>
+      <c r="D66" s="8">
+        <f>B46+B50+C50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="6" t="inlineStr">
+        <is>
+          <t>Savings / Goals (Section 3)</t>
+        </is>
+      </c>
+      <c r="B67" s="13" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C67" s="13">
+        <f>IFERROR(D67/D8,0)</f>
+        <v/>
+      </c>
+      <c r="D67" s="8">
+        <f>B35</f>
+        <v/>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="4" t="inlineStr">
-        <is>
-          <t>Bucket</t>
-        </is>
-      </c>
-      <c r="B69" s="5" t="inlineStr">
-        <is>
-          <t>Target %</t>
-        </is>
-      </c>
-      <c r="C69" s="5" t="inlineStr">
-        <is>
-          <t>Your %</t>
-        </is>
-      </c>
-      <c r="D69" s="5" t="inlineStr">
-        <is>
-          <t>Your $</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="6" t="inlineStr">
-        <is>
-          <t>Needs (Section 3)</t>
-        </is>
-      </c>
-      <c r="B70" s="11" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="C70" s="11">
-        <f>IFERROR(D70/D8,0)</f>
-        <v/>
-      </c>
-      <c r="D70" s="8">
-        <f>B29</f>
-        <v/>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="6" t="inlineStr">
-        <is>
-          <t>Wants (Sections 5 + 6)</t>
-        </is>
-      </c>
-      <c r="B71" s="11" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="C71" s="11">
-        <f>IFERROR(D71/D8,0)</f>
-        <v/>
-      </c>
-      <c r="D71" s="8">
-        <f>B51+B55+C55</f>
-        <v/>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="6" t="inlineStr">
-        <is>
-          <t>Savings / Goals (Section 4)</t>
-        </is>
-      </c>
-      <c r="B72" s="11" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="C72" s="11">
-        <f>IFERROR(D72/D8,0)</f>
-        <v/>
-      </c>
-      <c r="D72" s="8">
-        <f>B40</f>
-        <v/>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="12" t="inlineStr">
+      <c r="A69" s="12" t="inlineStr">
         <is>
           <t>With house + wedding goals active, it's normal for Savings/Goals to run above 20% and Wants below 30%.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="12">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A56:D56"/>
-    <mergeCell ref="A31:D31"/>
-    <mergeCell ref="A58:D58"/>
+    <mergeCell ref="A37:D37"/>
+    <mergeCell ref="A61:D61"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A53:D53"/>
-    <mergeCell ref="A68:D68"/>
+    <mergeCell ref="A69:D69"/>
     <mergeCell ref="A4:D4"/>
-    <mergeCell ref="A74:D74"/>
-    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A48:D48"/>
+    <mergeCell ref="A26:D26"/>
+    <mergeCell ref="A51:D51"/>
     <mergeCell ref="A10:D10"/>
-    <mergeCell ref="A42:D42"/>
-    <mergeCell ref="A13:D13"/>
-    <mergeCell ref="A66:D66"/>
+    <mergeCell ref="A63:D63"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Remove em dashes across repo
</commit_message>
<xml_diff>
--- a/01-current-budget/current-budget.xlsx
+++ b/01-current-budget/current-budget.xlsx
@@ -509,7 +509,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Current Monthly Budget — Kate &amp; Lucas</t>
+          <t>Current Monthly Budget - Kate &amp; Lucas</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>2. Fixed Needs — target ~50% of income</t>
+          <t>2. Fixed Needs - target ~50% of income</t>
         </is>
       </c>
     </row>
@@ -729,7 +729,7 @@
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>Subtotal — Needs</t>
+          <t>Subtotal - Needs</t>
         </is>
       </c>
       <c r="B24" s="10">
@@ -740,7 +740,7 @@
     <row r="26" ht="20" customHeight="1">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>3. Savings &amp; Goals — zero-based, prioritize explicitly</t>
+          <t>3. Savings &amp; Goals - zero-based, prioritize explicitly</t>
         </is>
       </c>
     </row>
@@ -827,7 +827,7 @@
     <row r="35">
       <c r="A35" s="9" t="inlineStr">
         <is>
-          <t>Subtotal — Savings &amp; Goals</t>
+          <t>Subtotal - Savings &amp; Goals</t>
         </is>
       </c>
       <c r="B35" s="10">
@@ -838,7 +838,7 @@
     <row r="37" ht="20" customHeight="1">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>4. Wants / Discretionary (shared) — target ~30% of income</t>
+          <t>4. Wants / Discretionary (shared) - target ~30% of income</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>Personal care (haircuts, gym, etc. — shared/household level)</t>
+          <t>Personal care (haircuts, gym, etc. - shared/household level)</t>
         </is>
       </c>
       <c r="B45" s="7" t="n"/>
@@ -925,7 +925,7 @@
     <row r="46">
       <c r="A46" s="9" t="inlineStr">
         <is>
-          <t>Subtotal — Shared Wants</t>
+          <t>Subtotal - Shared Wants</t>
         </is>
       </c>
       <c r="B46" s="10">
@@ -936,7 +936,7 @@
     <row r="48" ht="20" customHeight="1">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>5. Individual "Fun Money" — no itemizing, no questions asked</t>
+          <t>5. Individual "Fun Money" - no itemizing, no questions asked</t>
         </is>
       </c>
     </row>

</xml_diff>